<commit_message>
Add Track 7 (Amazon SP 21607 culpability), close all 21607 open questions, add SP 21607 entity list and screenshot
</commit_message>
<xml_diff>
--- a/master_violation_matrix.xlsx
+++ b/master_violation_matrix.xlsx
@@ -3310,7 +3310,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -4999,7 +4998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5138,6 +5137,46 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Amazon's direct culpability under DOT-SP 21607 (49 CFR 171.2(f))</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B0D97CRVM2, B0F62YLXK6 (both simultaneously print Amazon SP 21607 + R-134a on can)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SP 21607 marked but refrigerant hidden (Track 3 unauthorized marking still applies)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B0DT91W8NL, B0FFGQWXHG</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>